<commit_message>
Rebuild full product catalogue with guided interfaces
</commit_message>
<xml_diff>
--- a/02_excel_report_generator/reports/Sales_Performance_Report.xlsx
+++ b/02_excel_report_generator/reports/Sales_Performance_Report.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analysis" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw Data" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Report Information" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Executive Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Analysis" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Raw Data" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Report Information" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Executive Summary'!$A$1:$N$36</definedName>
@@ -260,7 +260,7 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <plotArea>
@@ -271,7 +271,7 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -321,7 +321,7 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="13"/>
   <chart>
     <plotArea>
@@ -331,14 +331,14 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -388,7 +388,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -403,9 +403,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -425,9 +425,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -777,7 +777,7 @@
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Executive report • Generated 12 July 2026 at 21:57</t>
+          <t>Executive report • Generated 13 July 2026 at 21:10</t>
         </is>
       </c>
     </row>
@@ -855,7 +855,7 @@
     <row r="36">
       <c r="A36" s="9" t="inlineStr">
         <is>
-          <t>Generated by Cooke Automation Systems  •  Excel Report Generator v1.0</t>
+          <t>Generated by Cooke Automation Systems  •  Excel Report Generator v2.0</t>
         </is>
       </c>
     </row>
@@ -2329,7 +2329,7 @@
       </c>
       <c r="B6" s="19" t="inlineStr">
         <is>
-          <t>1.0.0</t>
+          <t>2.0.0</t>
         </is>
       </c>
     </row>
@@ -2341,7 +2341,7 @@
       </c>
       <c r="B7" s="19" t="inlineStr">
         <is>
-          <t>sample_data/sample_sales.csv</t>
+          <t>/Users/deancooke/Desktop/Work/dean_automation_portfolio/02_excel_report_generator/sample_data/sample_sales.csv</t>
         </is>
       </c>
     </row>
@@ -2353,7 +2353,7 @@
       </c>
       <c r="B8" s="19" t="inlineStr">
         <is>
-          <t>12 July 2026 at 21:57</t>
+          <t>13 July 2026 at 21:10</t>
         </is>
       </c>
     </row>

</xml_diff>